<commit_message>
recreate testoutput and other datasets and add or update versioning metadata for all relevant datasets
</commit_message>
<xml_diff>
--- a/inst/testdata/examples_of_output/testoutput_ejam2excel_10pts_1miles.xlsx
+++ b/inst/testdata/examples_of_output/testoutput_ejam2excel_10pts_1miles.xlsx
@@ -1493,7 +1493,7 @@
     <t xml:space="preserve">area_sqmi</t>
   </si>
   <si>
-    <t xml:space="preserve">&lt;a href="https://ejanalysis.com", target="_blank"&gt;EJAM Site Report&lt;/a&gt;</t>
+    <t xml:space="preserve">&lt;a href="https://ejanalysis.com" target="_blank"&gt;EJAM Site Report&lt;/a&gt;</t>
   </si>
   <si>
     <t xml:space="preserve">https://pedp-ejscreen.azurewebsites.net/index.html</t>
@@ -1502,10 +1502,10 @@
     <t xml:space="preserve"/>
   </si>
   <si>
-    <t xml:space="preserve">&lt;a href="https://ejamapi-84652557241.us-central1.run.app/report?lat=37.64122&amp;lon=-122.410650&amp;buffer=1&amp;sitetype=latlon&amp;validate_regids=FALSE", target="_blank"&gt;EJAM Site Report&lt;/a&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;a href="https://pedp-ejscreen.azurewebsites.net/index.html?wherestr=37.64122,-122.41065", target="_blank"&gt;EJSCREEN&lt;/a&gt;</t>
+    <t xml:space="preserve">&lt;a href="https://ejamapi-84652557241.us-central1.run.app/report?lat=37.64122&amp;lon=-122.410650&amp;buffer=1&amp;sitetype=latlon&amp;validate_regids=FALSE" target="_blank"&gt;EJAM Site Report&lt;/a&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;a href="https://pedp-ejscreen.azurewebsites.net/index.html?wherestr=37.64122,-122.41065" target="_blank"&gt;EJSCREEN&lt;/a&gt;</t>
   </si>
   <si>
     <t xml:space="preserve">CA</t>
@@ -1514,10 +1514,10 @@
     <t xml:space="preserve">California</t>
   </si>
   <si>
-    <t xml:space="preserve">&lt;a href="https://ejamapi-84652557241.us-central1.run.app/report?lat=43.92249&amp;lon=%20-72.663705&amp;buffer=1&amp;sitetype=latlon&amp;validate_regids=FALSE", target="_blank"&gt;EJAM Site Report&lt;/a&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;a href="https://pedp-ejscreen.azurewebsites.net/index.html?wherestr=43.92249,-72.663705", target="_blank"&gt;EJSCREEN&lt;/a&gt;</t>
+    <t xml:space="preserve">&lt;a href="https://ejamapi-84652557241.us-central1.run.app/report?lat=43.92249&amp;lon=%20-72.663705&amp;buffer=1&amp;sitetype=latlon&amp;validate_regids=FALSE" target="_blank"&gt;EJAM Site Report&lt;/a&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;a href="https://pedp-ejscreen.azurewebsites.net/index.html?wherestr=43.92249,-72.663705" target="_blank"&gt;EJSCREEN&lt;/a&gt;</t>
   </si>
   <si>
     <t xml:space="preserve">VT</t>
@@ -1526,10 +1526,10 @@
     <t xml:space="preserve">Vermont</t>
   </si>
   <si>
-    <t xml:space="preserve">&lt;a href="https://ejamapi-84652557241.us-central1.run.app/report?lat=40.69351&amp;lon=%20-73.980020&amp;buffer=1&amp;sitetype=latlon&amp;validate_regids=FALSE", target="_blank"&gt;EJAM Site Report&lt;/a&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;a href="https://pedp-ejscreen.azurewebsites.net/index.html?wherestr=40.69351,-73.98002", target="_blank"&gt;EJSCREEN&lt;/a&gt;</t>
+    <t xml:space="preserve">&lt;a href="https://ejamapi-84652557241.us-central1.run.app/report?lat=40.69351&amp;lon=%20-73.980020&amp;buffer=1&amp;sitetype=latlon&amp;validate_regids=FALSE" target="_blank"&gt;EJAM Site Report&lt;/a&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;a href="https://pedp-ejscreen.azurewebsites.net/index.html?wherestr=40.69351,-73.98002" target="_blank"&gt;EJSCREEN&lt;/a&gt;</t>
   </si>
   <si>
     <t xml:space="preserve">NY</t>
@@ -1538,10 +1538,10 @@
     <t xml:space="preserve">New York</t>
   </si>
   <si>
-    <t xml:space="preserve">&lt;a href="https://ejamapi-84652557241.us-central1.run.app/report?lat=45.29520&amp;lon=%20-92.981840&amp;buffer=1&amp;sitetype=latlon&amp;validate_regids=FALSE", target="_blank"&gt;EJAM Site Report&lt;/a&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;a href="https://pedp-ejscreen.azurewebsites.net/index.html?wherestr=45.2952,-92.98184", target="_blank"&gt;EJSCREEN&lt;/a&gt;</t>
+    <t xml:space="preserve">&lt;a href="https://ejamapi-84652557241.us-central1.run.app/report?lat=45.29520&amp;lon=%20-92.981840&amp;buffer=1&amp;sitetype=latlon&amp;validate_regids=FALSE" target="_blank"&gt;EJAM Site Report&lt;/a&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;a href="https://pedp-ejscreen.azurewebsites.net/index.html?wherestr=45.2952,-92.98184" target="_blank"&gt;EJSCREEN&lt;/a&gt;</t>
   </si>
   <si>
     <t xml:space="preserve">MN</t>
@@ -1550,10 +1550,10 @@
     <t xml:space="preserve">Minnesota</t>
   </si>
   <si>
-    <t xml:space="preserve">&lt;a href="https://ejamapi-84652557241.us-central1.run.app/report?lat=39.43730&amp;lon=%20-74.723700&amp;buffer=1&amp;sitetype=latlon&amp;validate_regids=FALSE", target="_blank"&gt;EJAM Site Report&lt;/a&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;a href="https://pedp-ejscreen.azurewebsites.net/index.html?wherestr=39.4373,-74.7237", target="_blank"&gt;EJSCREEN&lt;/a&gt;</t>
+    <t xml:space="preserve">&lt;a href="https://ejamapi-84652557241.us-central1.run.app/report?lat=39.43730&amp;lon=%20-74.723700&amp;buffer=1&amp;sitetype=latlon&amp;validate_regids=FALSE" target="_blank"&gt;EJAM Site Report&lt;/a&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;a href="https://pedp-ejscreen.azurewebsites.net/index.html?wherestr=39.4373,-74.7237" target="_blank"&gt;EJSCREEN&lt;/a&gt;</t>
   </si>
   <si>
     <t xml:space="preserve">NJ</t>
@@ -1562,22 +1562,22 @@
     <t xml:space="preserve">New Jersey</t>
   </si>
   <si>
-    <t xml:space="preserve">&lt;a href="https://ejamapi-84652557241.us-central1.run.app/report?lat=45.67487&amp;lon=%20-94.815340&amp;buffer=1&amp;sitetype=latlon&amp;validate_regids=FALSE", target="_blank"&gt;EJAM Site Report&lt;/a&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;a href="https://pedp-ejscreen.azurewebsites.net/index.html?wherestr=45.67487,-94.81534", target="_blank"&gt;EJSCREEN&lt;/a&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;a href="https://ejamapi-84652557241.us-central1.run.app/report?lat=33.14865&amp;lon=-117.198950&amp;buffer=1&amp;sitetype=latlon&amp;validate_regids=FALSE", target="_blank"&gt;EJAM Site Report&lt;/a&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;a href="https://pedp-ejscreen.azurewebsites.net/index.html?wherestr=33.14865,-117.19895", target="_blank"&gt;EJSCREEN&lt;/a&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;a href="https://ejamapi-84652557241.us-central1.run.app/report?lat=34.01176&amp;lon=%20-80.954140&amp;buffer=1&amp;sitetype=latlon&amp;validate_regids=FALSE", target="_blank"&gt;EJAM Site Report&lt;/a&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;a href="https://pedp-ejscreen.azurewebsites.net/index.html?wherestr=34.01176,-80.95414", target="_blank"&gt;EJSCREEN&lt;/a&gt;</t>
+    <t xml:space="preserve">&lt;a href="https://ejamapi-84652557241.us-central1.run.app/report?lat=45.67487&amp;lon=%20-94.815340&amp;buffer=1&amp;sitetype=latlon&amp;validate_regids=FALSE" target="_blank"&gt;EJAM Site Report&lt;/a&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;a href="https://pedp-ejscreen.azurewebsites.net/index.html?wherestr=45.67487,-94.81534" target="_blank"&gt;EJSCREEN&lt;/a&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;a href="https://ejamapi-84652557241.us-central1.run.app/report?lat=33.14865&amp;lon=-117.198950&amp;buffer=1&amp;sitetype=latlon&amp;validate_regids=FALSE" target="_blank"&gt;EJAM Site Report&lt;/a&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;a href="https://pedp-ejscreen.azurewebsites.net/index.html?wherestr=33.14865,-117.19895" target="_blank"&gt;EJSCREEN&lt;/a&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;a href="https://ejamapi-84652557241.us-central1.run.app/report?lat=34.01176&amp;lon=%20-80.954140&amp;buffer=1&amp;sitetype=latlon&amp;validate_regids=FALSE" target="_blank"&gt;EJAM Site Report&lt;/a&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;a href="https://pedp-ejscreen.azurewebsites.net/index.html?wherestr=34.01176,-80.95414" target="_blank"&gt;EJSCREEN&lt;/a&gt;</t>
   </si>
   <si>
     <t xml:space="preserve">SC</t>
@@ -1586,10 +1586,10 @@
     <t xml:space="preserve">South Carolina</t>
   </si>
   <si>
-    <t xml:space="preserve">&lt;a href="https://ejamapi-84652557241.us-central1.run.app/report?lat=43.01026&amp;lon=%20-89.459520&amp;buffer=1&amp;sitetype=latlon&amp;validate_regids=FALSE", target="_blank"&gt;EJAM Site Report&lt;/a&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;a href="https://pedp-ejscreen.azurewebsites.net/index.html?wherestr=43.01026,-89.45952", target="_blank"&gt;EJSCREEN&lt;/a&gt;</t>
+    <t xml:space="preserve">&lt;a href="https://ejamapi-84652557241.us-central1.run.app/report?lat=43.01026&amp;lon=%20-89.459520&amp;buffer=1&amp;sitetype=latlon&amp;validate_regids=FALSE" target="_blank"&gt;EJAM Site Report&lt;/a&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;a href="https://pedp-ejscreen.azurewebsites.net/index.html?wherestr=43.01026,-89.45952" target="_blank"&gt;EJSCREEN&lt;/a&gt;</t>
   </si>
   <si>
     <t xml:space="preserve">WI</t>
@@ -1598,10 +1598,10 @@
     <t xml:space="preserve">Wisconsin</t>
   </si>
   <si>
-    <t xml:space="preserve">&lt;a href="https://ejamapi-84652557241.us-central1.run.app/report?lat=40.74625&amp;lon=%20-74.259550&amp;buffer=1&amp;sitetype=latlon&amp;validate_regids=FALSE", target="_blank"&gt;EJAM Site Report&lt;/a&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;a href="https://pedp-ejscreen.azurewebsites.net/index.html?wherestr=40.74625,-74.25955", target="_blank"&gt;EJSCREEN&lt;/a&gt;</t>
+    <t xml:space="preserve">&lt;a href="https://ejamapi-84652557241.us-central1.run.app/report?lat=40.74625&amp;lon=%20-74.259550&amp;buffer=1&amp;sitetype=latlon&amp;validate_regids=FALSE" target="_blank"&gt;EJAM Site Report&lt;/a&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;a href="https://pedp-ejscreen.azurewebsites.net/index.html?wherestr=40.74625,-74.25955" target="_blank"&gt;EJSCREEN&lt;/a&gt;</t>
   </si>
   <si>
     <t xml:space="preserve">value</t>

</xml_diff>

<commit_message>
Health rows as whole percents; Climate after Poverty; compact footnote
- New pct_as_points_ejamit column in map_headernames: rateheartdisease,
  rateasthma, ratecancer (+ avg./state.avg. rows) are stored as 0-100
  percentage points, so format_ejamit_columns() now shows them with a % sign
  and no x100 rescaling ("10%" not "9.90"), decimals set to 0 like other
  percent rows; ejam2excel styling gives them a literal % suffix instead of
  the x100 "0%" percent style (which would have displayed 387% for heart
  disease). Demog.Index and other rows unaffected.
- Climate section moved up to sit right after Poverty (following the
  flagged-areas "% of These Residents..." rows); Other Totals stays last.
- Report footnote block uses compact line spacing (line-height 1.25, small
  margins).
- map_headernames.rda + all report/excel testoutputs regenerated; NEWS + man
  updated.

Addresses the follow-up review comments on #444.
</commit_message>
<xml_diff>
--- a/inst/testdata/examples_of_output/testoutput_ejam2excel_10pts_1miles.xlsx
+++ b/inst/testdata/examples_of_output/testoutput_ejam2excel_10pts_1miles.xlsx
@@ -5191,8 +5191,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="11">
-    <numFmt numFmtId="167" formatCode="#,###,###"/>
+  <numFmts count="12">
+    <numFmt numFmtId="168" formatCode="#,###,###"/>
     <numFmt numFmtId="169" formatCode="#,###,##0.0"/>
     <numFmt numFmtId="171" formatCode="#,###,##0.00"/>
     <numFmt numFmtId="172" formatCode="#,###,##0.000"/>
@@ -5201,8 +5201,9 @@
     <numFmt numFmtId="175" formatCode="#,##0.0"/>
     <numFmt numFmtId="176" formatCode="#0"/>
     <numFmt numFmtId="177" formatCode="0%"/>
-    <numFmt numFmtId="178" formatCode="#,###,###"/>
-    <numFmt numFmtId="179" formatCode="$#,##0"/>
+    <numFmt numFmtId="178" formatCode="0&quot;%&quot;"/>
+    <numFmt numFmtId="179" formatCode="#,###,###"/>
+    <numFmt numFmtId="180" formatCode="$#,##0"/>
   </numFmts>
   <fonts count="4">
     <font>
@@ -5360,7 +5361,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -5432,7 +5433,7 @@
     <xf numFmtId="0" fontId="2" fillId="22" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1"/>
+    <xf numFmtId="168" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1"/>
     <xf numFmtId="169" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1"/>
     <xf numFmtId="171" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1"/>
     <xf numFmtId="172" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1"/>
@@ -5443,6 +5444,7 @@
     <xf numFmtId="177" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1"/>
     <xf numFmtId="178" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1"/>
     <xf numFmtId="179" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1"/>
+    <xf numFmtId="180" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -8192,7 +8194,7 @@
       <c r="E2" t="s">
         <v>17</v>
       </c>
-      <c r="F2" s="34" t="n">
+      <c r="F2" s="35" t="n">
         <v>14025.6</v>
       </c>
       <c r="G2" t="n">
@@ -8678,7 +8680,7 @@
       <c r="FK2" s="33" t="n">
         <v>0.463471896936268</v>
       </c>
-      <c r="FL2" s="35" t="n">
+      <c r="FL2" s="36" t="n">
         <v>50062.3361863197</v>
       </c>
       <c r="FM2" s="33" t="n">
@@ -8759,13 +8761,13 @@
       <c r="GL2" s="33" t="n">
         <v>0.179515638237509</v>
       </c>
-      <c r="GM2" s="33" t="n">
+      <c r="GM2" s="34" t="n">
         <v>4.09841464967071</v>
       </c>
-      <c r="GN2" s="27" t="n">
+      <c r="GN2" s="34" t="n">
         <v>8.64702294436022</v>
       </c>
-      <c r="GO2" s="27" t="n">
+      <c r="GO2" s="34" t="n">
         <v>4.84812175044326</v>
       </c>
       <c r="GP2" s="25" t="n">
@@ -9176,13 +9178,13 @@
       <c r="LU2" s="33" t="n">
         <v>0.195319647024096</v>
       </c>
-      <c r="LV2" s="33" t="n">
+      <c r="LV2" s="34" t="n">
         <v>5.78866112415659</v>
       </c>
-      <c r="LW2" s="25" t="n">
+      <c r="LW2" s="34" t="n">
         <v>10.3142467897866</v>
       </c>
-      <c r="LX2" s="26" t="n">
+      <c r="LX2" s="34" t="n">
         <v>6.44134924160715</v>
       </c>
       <c r="LY2" s="33" t="n">
@@ -9293,13 +9295,13 @@
       <c r="NH2" s="33" t="n">
         <v>0.17650023381035</v>
       </c>
-      <c r="NI2" s="33" t="n">
+      <c r="NI2" s="34" t="n">
         <v>4.76004234961966</v>
       </c>
-      <c r="NJ2" s="26" t="n">
+      <c r="NJ2" s="34" t="n">
         <v>9.5911614775312</v>
       </c>
-      <c r="NK2" s="26" t="n">
+      <c r="NK2" s="34" t="n">
         <v>5.56444592580973</v>
       </c>
       <c r="NL2" s="33" t="n">
@@ -10243,7 +10245,7 @@
       <c r="E3" t="s">
         <v>17</v>
       </c>
-      <c r="F3" s="34" t="n">
+      <c r="F3" s="35" t="n">
         <v>1584.6</v>
       </c>
       <c r="G3" t="n">
@@ -10711,7 +10713,7 @@
       <c r="FK3" s="33" t="n">
         <v>0.484920385823632</v>
       </c>
-      <c r="FL3" s="35" t="n">
+      <c r="FL3" s="36" t="n">
         <v>32205.5185662568</v>
       </c>
       <c r="FM3" s="33" t="n">
@@ -10784,13 +10786,13 @@
       <c r="GL3" s="33" t="n">
         <v>0.17948717948718</v>
       </c>
-      <c r="GM3" s="33" t="n">
+      <c r="GM3" s="34" t="n">
         <v>5.7</v>
       </c>
-      <c r="GN3" s="27" t="n">
+      <c r="GN3" s="34" t="n">
         <v>10.7</v>
       </c>
-      <c r="GO3" s="27" t="n">
+      <c r="GO3" s="34" t="n">
         <v>7.2</v>
       </c>
       <c r="GP3" s="25" t="n">
@@ -11201,13 +11203,13 @@
       <c r="LU3" s="33" t="n">
         <v>0.195319647024096</v>
       </c>
-      <c r="LV3" s="33" t="n">
+      <c r="LV3" s="34" t="n">
         <v>5.78866112415659</v>
       </c>
-      <c r="LW3" s="25" t="n">
+      <c r="LW3" s="34" t="n">
         <v>10.3142467897866</v>
       </c>
-      <c r="LX3" s="26" t="n">
+      <c r="LX3" s="34" t="n">
         <v>6.44134924160715</v>
       </c>
       <c r="LY3" s="33" t="n">
@@ -11318,13 +11320,13 @@
       <c r="NH3" s="33" t="n">
         <v>0.169786003470214</v>
       </c>
-      <c r="NI3" s="33" t="n">
+      <c r="NI3" s="34" t="n">
         <v>5.68642201834863</v>
       </c>
-      <c r="NJ3" s="26" t="n">
+      <c r="NJ3" s="34" t="n">
         <v>11.0229357798165</v>
       </c>
-      <c r="NK3" s="26" t="n">
+      <c r="NK3" s="34" t="n">
         <v>7.23633027522936</v>
       </c>
       <c r="NL3" s="33" t="n">
@@ -12252,7 +12254,7 @@
       <c r="E4" t="s">
         <v>17</v>
       </c>
-      <c r="F4" s="34" t="n">
+      <c r="F4" s="35" t="n">
         <v>137834.8</v>
       </c>
       <c r="G4" t="n">
@@ -12738,7 +12740,7 @@
       <c r="FK4" s="33" t="n">
         <v>0.537863956387226</v>
       </c>
-      <c r="FL4" s="35" t="n">
+      <c r="FL4" s="36" t="n">
         <v>93647.6305037285</v>
       </c>
       <c r="FM4" s="33" t="n">
@@ -12819,13 +12821,13 @@
       <c r="GL4" s="33" t="n">
         <v>0.173235590729745</v>
       </c>
-      <c r="GM4" s="33" t="n">
+      <c r="GM4" s="34" t="n">
         <v>3.48011227084465</v>
       </c>
-      <c r="GN4" s="27" t="n">
+      <c r="GN4" s="34" t="n">
         <v>10.0431313115477</v>
       </c>
-      <c r="GO4" s="27" t="n">
+      <c r="GO4" s="34" t="n">
         <v>4.51127485960828</v>
       </c>
       <c r="GP4" s="25" t="n">
@@ -13236,13 +13238,13 @@
       <c r="LU4" s="33" t="n">
         <v>0.195319647024096</v>
       </c>
-      <c r="LV4" s="33" t="n">
+      <c r="LV4" s="34" t="n">
         <v>5.78866112415659</v>
       </c>
-      <c r="LW4" s="25" t="n">
+      <c r="LW4" s="34" t="n">
         <v>10.3142467897866</v>
       </c>
-      <c r="LX4" s="26" t="n">
+      <c r="LX4" s="34" t="n">
         <v>6.44134924160715</v>
       </c>
       <c r="LY4" s="33" t="n">
@@ -13353,13 +13355,13 @@
       <c r="NH4" s="33" t="n">
         <v>0.174060685726804</v>
       </c>
-      <c r="NI4" s="33" t="n">
+      <c r="NI4" s="34" t="n">
         <v>5.4719139370585</v>
       </c>
-      <c r="NJ4" s="26" t="n">
+      <c r="NJ4" s="34" t="n">
         <v>10.9509762363521</v>
       </c>
-      <c r="NK4" s="26" t="n">
+      <c r="NK4" s="34" t="n">
         <v>6.32426461143226</v>
       </c>
       <c r="NL4" s="33" t="n">
@@ -14303,7 +14305,7 @@
       <c r="E5" t="s">
         <v>17</v>
       </c>
-      <c r="F5" s="34" t="n">
+      <c r="F5" s="35" t="n">
         <v>1906</v>
       </c>
       <c r="G5" t="n">
@@ -14789,7 +14791,7 @@
       <c r="FK5" s="33" t="n">
         <v>0.507578400071129</v>
       </c>
-      <c r="FL5" s="35" t="n">
+      <c r="FL5" s="36" t="n">
         <v>43031.6277237555</v>
       </c>
       <c r="FM5" s="33" t="n">
@@ -14870,13 +14872,13 @@
       <c r="GL5" s="33" t="n">
         <v>0.182475225109122</v>
       </c>
-      <c r="GM5" s="33" t="n">
+      <c r="GM5" s="34" t="n">
         <v>4.69006520935133</v>
       </c>
-      <c r="GN5" s="27" t="n">
+      <c r="GN5" s="34" t="n">
         <v>9.27855218026365</v>
       </c>
-      <c r="GO5" s="27" t="n">
+      <c r="GO5" s="34" t="n">
         <v>6.52223693895585</v>
       </c>
       <c r="GP5" s="25" t="n">
@@ -15287,13 +15289,13 @@
       <c r="LU5" s="33" t="n">
         <v>0.195319647024096</v>
       </c>
-      <c r="LV5" s="33" t="n">
+      <c r="LV5" s="34" t="n">
         <v>5.78866112415659</v>
       </c>
-      <c r="LW5" s="25" t="n">
+      <c r="LW5" s="34" t="n">
         <v>10.3142467897866</v>
       </c>
-      <c r="LX5" s="26" t="n">
+      <c r="LX5" s="34" t="n">
         <v>6.44134924160715</v>
       </c>
       <c r="LY5" s="33" t="n">
@@ -15404,13 +15406,13 @@
       <c r="NH5" s="33" t="n">
         <v>0.173092206559966</v>
       </c>
-      <c r="NI5" s="33" t="n">
+      <c r="NI5" s="34" t="n">
         <v>5.19868193604147</v>
       </c>
-      <c r="NJ5" s="26" t="n">
+      <c r="NJ5" s="34" t="n">
         <v>9.54753673293002</v>
       </c>
-      <c r="NK5" s="26" t="n">
+      <c r="NK5" s="34" t="n">
         <v>6.69461970613658</v>
       </c>
       <c r="NL5" s="33" t="n">
@@ -16354,7 +16356,7 @@
       <c r="E6" t="s">
         <v>17</v>
       </c>
-      <c r="F6" s="34" t="n">
+      <c r="F6" s="35" t="n">
         <v>1519.5</v>
       </c>
       <c r="G6" t="n">
@@ -16824,7 +16826,7 @@
       <c r="FK6" s="33" t="n">
         <v>0.499597646556648</v>
       </c>
-      <c r="FL6" s="35" t="n">
+      <c r="FL6" s="36" t="n">
         <v>57591.9650491898</v>
       </c>
       <c r="FM6" s="33" t="n">
@@ -16897,13 +16899,13 @@
       <c r="GL6" s="33" t="n">
         <v>0.19291242929342</v>
       </c>
-      <c r="GM6" s="33" t="n">
+      <c r="GM6" s="34" t="n">
         <v>5.73026119122173</v>
       </c>
-      <c r="GN6" s="27" t="n">
+      <c r="GN6" s="34" t="n">
         <v>9.76635700435717</v>
       </c>
-      <c r="GO6" s="27" t="n">
+      <c r="GO6" s="34" t="n">
         <v>7.2869685277176</v>
       </c>
       <c r="GP6" s="25" t="n">
@@ -17314,13 +17316,13 @@
       <c r="LU6" s="33" t="n">
         <v>0.195319647024096</v>
       </c>
-      <c r="LV6" s="33" t="n">
+      <c r="LV6" s="34" t="n">
         <v>5.78866112415659</v>
       </c>
-      <c r="LW6" s="25" t="n">
+      <c r="LW6" s="34" t="n">
         <v>10.3142467897866</v>
       </c>
-      <c r="LX6" s="26" t="n">
+      <c r="LX6" s="34" t="n">
         <v>6.44134924160715</v>
       </c>
       <c r="LY6" s="33" t="n">
@@ -17431,13 +17433,13 @@
       <c r="NH6" s="33" t="n">
         <v>0.180930565730564</v>
       </c>
-      <c r="NI6" s="33" t="n">
+      <c r="NI6" s="34" t="n">
         <v>5.27495307967926</v>
       </c>
-      <c r="NJ6" s="26" t="n">
+      <c r="NJ6" s="34" t="n">
         <v>9.51977478246032</v>
       </c>
-      <c r="NK6" s="26" t="n">
+      <c r="NK6" s="34" t="n">
         <v>6.62590001706193</v>
       </c>
       <c r="NL6" s="33" t="n">
@@ -18365,7 +18367,7 @@
       <c r="E7" t="s">
         <v>17</v>
       </c>
-      <c r="F7" s="34" t="n">
+      <c r="F7" s="35" t="n">
         <v>3620.3</v>
       </c>
       <c r="G7" t="n">
@@ -18851,7 +18853,7 @@
       <c r="FK7" s="33" t="n">
         <v>0.46919249986657</v>
       </c>
-      <c r="FL7" s="35" t="n">
+      <c r="FL7" s="36" t="n">
         <v>34267.9740512576</v>
       </c>
       <c r="FM7" s="33" t="n">
@@ -18932,13 +18934,13 @@
       <c r="GL7" s="33" t="n">
         <v>0.154036213058758</v>
       </c>
-      <c r="GM7" s="33" t="n">
+      <c r="GM7" s="34" t="n">
         <v>6.54940880274376</v>
       </c>
-      <c r="GN7" s="27" t="n">
+      <c r="GN7" s="34" t="n">
         <v>9.1797635210975</v>
       </c>
-      <c r="GO7" s="27" t="n">
+      <c r="GO7" s="34" t="n">
         <v>7.9797635210975</v>
       </c>
       <c r="GP7" s="25" t="n">
@@ -19349,13 +19351,13 @@
       <c r="LU7" s="33" t="n">
         <v>0.195319647024096</v>
       </c>
-      <c r="LV7" s="33" t="n">
+      <c r="LV7" s="34" t="n">
         <v>5.78866112415659</v>
       </c>
-      <c r="LW7" s="25" t="n">
+      <c r="LW7" s="34" t="n">
         <v>10.3142467897866</v>
       </c>
-      <c r="LX7" s="26" t="n">
+      <c r="LX7" s="34" t="n">
         <v>6.44134924160715</v>
       </c>
       <c r="LY7" s="33" t="n">
@@ -19466,13 +19468,13 @@
       <c r="NH7" s="33" t="n">
         <v>0.173092206559966</v>
       </c>
-      <c r="NI7" s="33" t="n">
+      <c r="NI7" s="34" t="n">
         <v>5.19868193604147</v>
       </c>
-      <c r="NJ7" s="26" t="n">
+      <c r="NJ7" s="34" t="n">
         <v>9.54753673293002</v>
       </c>
-      <c r="NK7" s="26" t="n">
+      <c r="NK7" s="34" t="n">
         <v>6.69461970613658</v>
       </c>
       <c r="NL7" s="33" t="n">
@@ -20416,7 +20418,7 @@
       <c r="E8" t="s">
         <v>17</v>
       </c>
-      <c r="F8" s="34" t="n">
+      <c r="F8" s="35" t="n">
         <v>14810.4</v>
       </c>
       <c r="G8" t="n">
@@ -20902,7 +20904,7 @@
       <c r="FK8" s="33" t="n">
         <v>0.514527154955763</v>
       </c>
-      <c r="FL8" s="35" t="n">
+      <c r="FL8" s="36" t="n">
         <v>31106.1531097072</v>
       </c>
       <c r="FM8" s="33" t="n">
@@ -20983,13 +20985,13 @@
       <c r="GL8" s="33" t="n">
         <v>0.159031651949576</v>
       </c>
-      <c r="GM8" s="33" t="n">
+      <c r="GM8" s="34" t="n">
         <v>5.0175293795214</v>
       </c>
-      <c r="GN8" s="27" t="n">
+      <c r="GN8" s="34" t="n">
         <v>10.0809724159956</v>
       </c>
-      <c r="GO8" s="27" t="n">
+      <c r="GO8" s="34" t="n">
         <v>4.93121936668601</v>
       </c>
       <c r="GP8" s="25" t="n">
@@ -21400,13 +21402,13 @@
       <c r="LU8" s="33" t="n">
         <v>0.195319647024096</v>
       </c>
-      <c r="LV8" s="33" t="n">
+      <c r="LV8" s="34" t="n">
         <v>5.78866112415659</v>
       </c>
-      <c r="LW8" s="25" t="n">
+      <c r="LW8" s="34" t="n">
         <v>10.3142467897866</v>
       </c>
-      <c r="LX8" s="26" t="n">
+      <c r="LX8" s="34" t="n">
         <v>6.44134924160715</v>
       </c>
       <c r="LY8" s="33" t="n">
@@ -21517,13 +21519,13 @@
       <c r="NH8" s="33" t="n">
         <v>0.17650023381035</v>
       </c>
-      <c r="NI8" s="33" t="n">
+      <c r="NI8" s="34" t="n">
         <v>4.76004234961966</v>
       </c>
-      <c r="NJ8" s="26" t="n">
+      <c r="NJ8" s="34" t="n">
         <v>9.5911614775312</v>
       </c>
-      <c r="NK8" s="26" t="n">
+      <c r="NK8" s="34" t="n">
         <v>5.56444592580973</v>
       </c>
       <c r="NL8" s="33" t="n">
@@ -22467,7 +22469,7 @@
       <c r="E9" t="s">
         <v>17</v>
       </c>
-      <c r="F9" s="34" t="n">
+      <c r="F9" s="35" t="n">
         <v>3935.3</v>
       </c>
       <c r="G9" t="n">
@@ -22953,7 +22955,7 @@
       <c r="FK9" s="33" t="n">
         <v>0.444238925811023</v>
       </c>
-      <c r="FL9" s="35" t="n">
+      <c r="FL9" s="36" t="n">
         <v>60221.7342041206</v>
       </c>
       <c r="FM9" s="33" t="n">
@@ -23034,13 +23036,13 @@
       <c r="GL9" s="33" t="n">
         <v>0.166075136088855</v>
       </c>
-      <c r="GM9" s="33" t="n">
+      <c r="GM9" s="34" t="n">
         <v>3.69512513816529</v>
       </c>
-      <c r="GN9" s="27" t="n">
+      <c r="GN9" s="34" t="n">
         <v>8.31521514727601</v>
       </c>
-      <c r="GO9" s="27" t="n">
+      <c r="GO9" s="34" t="n">
         <v>5.75040746621621</v>
       </c>
       <c r="GP9" s="25" t="n">
@@ -23451,13 +23453,13 @@
       <c r="LU9" s="33" t="n">
         <v>0.195319647024096</v>
       </c>
-      <c r="LV9" s="33" t="n">
+      <c r="LV9" s="34" t="n">
         <v>5.78866112415659</v>
       </c>
-      <c r="LW9" s="25" t="n">
+      <c r="LW9" s="34" t="n">
         <v>10.3142467897866</v>
       </c>
-      <c r="LX9" s="26" t="n">
+      <c r="LX9" s="34" t="n">
         <v>6.44134924160715</v>
       </c>
       <c r="LY9" s="33" t="n">
@@ -23568,13 +23570,13 @@
       <c r="NH9" s="33" t="n">
         <v>0.214244555155618</v>
       </c>
-      <c r="NI9" s="33" t="n">
+      <c r="NI9" s="34" t="n">
         <v>6.17180851063831</v>
       </c>
-      <c r="NJ9" s="26" t="n">
+      <c r="NJ9" s="34" t="n">
         <v>9.9034278959811</v>
       </c>
-      <c r="NK9" s="26" t="n">
+      <c r="NK9" s="34" t="n">
         <v>6.59175531914892</v>
       </c>
       <c r="NL9" s="33" t="n">
@@ -24518,7 +24520,7 @@
       <c r="E10" t="s">
         <v>17</v>
       </c>
-      <c r="F10" s="34" t="n">
+      <c r="F10" s="35" t="n">
         <v>4183.8</v>
       </c>
       <c r="G10" t="n">
@@ -25004,7 +25006,7 @@
       <c r="FK10" s="33" t="n">
         <v>0.47672304254243</v>
       </c>
-      <c r="FL10" s="35" t="n">
+      <c r="FL10" s="36" t="n">
         <v>72255.0104056962</v>
       </c>
       <c r="FM10" s="33" t="n">
@@ -25085,13 +25087,13 @@
       <c r="GL10" s="33" t="n">
         <v>0.165603327574603</v>
       </c>
-      <c r="GM10" s="33" t="n">
+      <c r="GM10" s="34" t="n">
         <v>3.9932669515546</v>
       </c>
-      <c r="GN10" s="27" t="n">
+      <c r="GN10" s="34" t="n">
         <v>10.2802406377357</v>
       </c>
-      <c r="GO10" s="27" t="n">
+      <c r="GO10" s="34" t="n">
         <v>6.09743806051871</v>
       </c>
       <c r="GP10" s="25" t="n">
@@ -25502,13 +25504,13 @@
       <c r="LU10" s="33" t="n">
         <v>0.195319647024096</v>
       </c>
-      <c r="LV10" s="33" t="n">
+      <c r="LV10" s="34" t="n">
         <v>5.78866112415659</v>
       </c>
-      <c r="LW10" s="25" t="n">
+      <c r="LW10" s="34" t="n">
         <v>10.3142467897866</v>
       </c>
-      <c r="LX10" s="26" t="n">
+      <c r="LX10" s="34" t="n">
         <v>6.44134924160715</v>
       </c>
       <c r="LY10" s="33" t="n">
@@ -25619,13 +25621,13 @@
       <c r="NH10" s="33" t="n">
         <v>0.188286534241179</v>
       </c>
-      <c r="NI10" s="33" t="n">
+      <c r="NI10" s="34" t="n">
         <v>5.55841455490577</v>
       </c>
-      <c r="NJ10" s="26" t="n">
+      <c r="NJ10" s="34" t="n">
         <v>10.7292830842538</v>
       </c>
-      <c r="NK10" s="26" t="n">
+      <c r="NK10" s="34" t="n">
         <v>6.95029239766081</v>
       </c>
       <c r="NL10" s="33" t="n">
@@ -26569,7 +26571,7 @@
       <c r="E11" t="s">
         <v>17</v>
       </c>
-      <c r="F11" s="34" t="n">
+      <c r="F11" s="35" t="n">
         <v>28896.7</v>
       </c>
       <c r="G11" t="n">
@@ -27055,7 +27057,7 @@
       <c r="FK11" s="33" t="n">
         <v>0.495678256567942</v>
       </c>
-      <c r="FL11" s="35" t="n">
+      <c r="FL11" s="36" t="n">
         <v>61244.0406923008</v>
       </c>
       <c r="FM11" s="33" t="n">
@@ -27136,13 +27138,13 @@
       <c r="GL11" s="33" t="n">
         <v>0.14982163881401</v>
       </c>
-      <c r="GM11" s="33" t="n">
+      <c r="GM11" s="34" t="n">
         <v>4.44187763821409</v>
       </c>
-      <c r="GN11" s="27" t="n">
+      <c r="GN11" s="34" t="n">
         <v>9.84789323887864</v>
       </c>
-      <c r="GO11" s="27" t="n">
+      <c r="GO11" s="34" t="n">
         <v>5.74163374613537</v>
       </c>
       <c r="GP11" s="25" t="n">
@@ -27553,13 +27555,13 @@
       <c r="LU11" s="33" t="n">
         <v>0.195319647024096</v>
       </c>
-      <c r="LV11" s="33" t="n">
+      <c r="LV11" s="34" t="n">
         <v>5.78866112415659</v>
       </c>
-      <c r="LW11" s="25" t="n">
+      <c r="LW11" s="34" t="n">
         <v>10.3142467897866</v>
       </c>
-      <c r="LX11" s="26" t="n">
+      <c r="LX11" s="34" t="n">
         <v>6.44134924160715</v>
       </c>
       <c r="LY11" s="33" t="n">
@@ -27670,13 +27672,13 @@
       <c r="NH11" s="33" t="n">
         <v>0.180930565730564</v>
       </c>
-      <c r="NI11" s="33" t="n">
+      <c r="NI11" s="34" t="n">
         <v>5.27495307967926</v>
       </c>
-      <c r="NJ11" s="26" t="n">
+      <c r="NJ11" s="34" t="n">
         <v>9.51977478246032</v>
       </c>
-      <c r="NK11" s="26" t="n">
+      <c r="NK11" s="34" t="n">
         <v>6.62590001706193</v>
       </c>
       <c r="NL11" s="33" t="n">
@@ -31725,7 +31727,7 @@
       <c r="E2" t="s">
         <v>17</v>
       </c>
-      <c r="F2" s="34" t="n">
+      <c r="F2" s="35" t="n">
         <v>212317</v>
       </c>
       <c r="G2"/>
@@ -32201,7 +32203,7 @@
       <c r="FK2" s="33" t="n">
         <v>0.520528229254851</v>
       </c>
-      <c r="FL2" s="35" t="n">
+      <c r="FL2" s="36" t="n">
         <v>78770.1299499313</v>
       </c>
       <c r="FM2" s="33" t="n">
@@ -32282,13 +32284,13 @@
       <c r="GL2" s="33" t="n">
         <v>0.169039787917734</v>
       </c>
-      <c r="GM2" s="33" t="n">
+      <c r="GM2" s="34" t="n">
         <v>3.86906513605095</v>
       </c>
-      <c r="GN2" s="27" t="n">
+      <c r="GN2" s="34" t="n">
         <v>9.88095400580117</v>
       </c>
-      <c r="GO2" s="27" t="n">
+      <c r="GO2" s="34" t="n">
         <v>4.90162453569761</v>
       </c>
       <c r="GP2" s="25" t="n">
@@ -32699,13 +32701,13 @@
       <c r="LU2" s="33" t="n">
         <v>0.195319647024096</v>
       </c>
-      <c r="LV2" s="33" t="n">
+      <c r="LV2" s="34" t="n">
         <v>5.78866112415659</v>
       </c>
-      <c r="LW2" s="25" t="n">
+      <c r="LW2" s="34" t="n">
         <v>10.3142467897866</v>
       </c>
-      <c r="LX2" s="26" t="n">
+      <c r="LX2" s="34" t="n">
         <v>6.44134924160715</v>
       </c>
       <c r="LY2" s="33" t="n">
@@ -32816,13 +32818,13 @@
       <c r="NH2" s="33" t="n">
         <v>0.176344206929354</v>
       </c>
-      <c r="NI2" s="33" t="n">
+      <c r="NI2" s="34" t="n">
         <v>5.35618045350864</v>
       </c>
-      <c r="NJ2" s="26" t="n">
+      <c r="NJ2" s="34" t="n">
         <v>10.5014829528372</v>
       </c>
-      <c r="NK2" s="26" t="n">
+      <c r="NK2" s="34" t="n">
         <v>6.29802203571255</v>
       </c>
       <c r="NL2" s="33" t="n">

</xml_diff>

<commit_message>
Apply pct_as_points excel numFmt in one place only
Per Copilot review on #444: the per-decimals styling loop now skips
pct_as_points_ejamit columns entirely, so their literal-% number format is
applied only by the dedicated pctpoints_style block. Verified each affected
column carries exactly one numFmt (value and US/State-average columns: 0"%";
ratio columns unchanged at #,##0.0; percentiles #0). Excel testoutputs
regenerated; test-ejam2excel passes.
</commit_message>
<xml_diff>
--- a/inst/testdata/examples_of_output/testoutput_ejam2excel_10pts_1miles.xlsx
+++ b/inst/testdata/examples_of_output/testoutput_ejam2excel_10pts_1miles.xlsx
@@ -5192,18 +5192,18 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="12">
-    <numFmt numFmtId="168" formatCode="#,###,###"/>
-    <numFmt numFmtId="169" formatCode="#,###,##0.0"/>
-    <numFmt numFmtId="171" formatCode="#,###,##0.00"/>
-    <numFmt numFmtId="172" formatCode="#,###,##0.000"/>
+    <numFmt numFmtId="167" formatCode="#,###,###"/>
+    <numFmt numFmtId="168" formatCode="#,###,##0.0"/>
+    <numFmt numFmtId="170" formatCode="#,###,##0.00"/>
+    <numFmt numFmtId="171" formatCode="#,###,##0.000"/>
+    <numFmt numFmtId="172" formatCode="#,##0.00"/>
     <numFmt numFmtId="173" formatCode="#,##0.00"/>
-    <numFmt numFmtId="174" formatCode="#,##0.00"/>
-    <numFmt numFmtId="175" formatCode="#,##0.0"/>
-    <numFmt numFmtId="176" formatCode="#0"/>
-    <numFmt numFmtId="177" formatCode="0%"/>
-    <numFmt numFmtId="178" formatCode="0&quot;%&quot;"/>
-    <numFmt numFmtId="179" formatCode="#,###,###"/>
-    <numFmt numFmtId="180" formatCode="$#,##0"/>
+    <numFmt numFmtId="174" formatCode="#,##0.0"/>
+    <numFmt numFmtId="175" formatCode="#0"/>
+    <numFmt numFmtId="176" formatCode="0%"/>
+    <numFmt numFmtId="177" formatCode="0&quot;%&quot;"/>
+    <numFmt numFmtId="178" formatCode="#,###,###"/>
+    <numFmt numFmtId="179" formatCode="$#,##0"/>
   </numFmts>
   <fonts count="4">
     <font>
@@ -5433,8 +5433,9 @@
     <xf numFmtId="0" fontId="2" fillId="22" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="167" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1"/>
     <xf numFmtId="168" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1"/>
-    <xf numFmtId="169" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1"/>
+    <xf numFmtId="170" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1"/>
     <xf numFmtId="171" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1"/>
     <xf numFmtId="172" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1"/>
     <xf numFmtId="173" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1"/>
@@ -5444,7 +5445,6 @@
     <xf numFmtId="177" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1"/>
     <xf numFmtId="178" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1"/>
     <xf numFmtId="179" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1"/>
-    <xf numFmtId="180" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>

</xml_diff>